<commit_message>
adiciona o fluxo login capaz de atuar no onedrive
</commit_message>
<xml_diff>
--- a/data/remanejamento.xlsx
+++ b/data/remanejamento.xlsx
@@ -1,24 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\guilhermemelof\code\splor-mg\siafi-automacao-cota\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34E0ED5D-E8DD-4DD3-B23B-73A4BB4F7D9D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B4C85F4-DE41-4A33-B9A0-48623C19BC30}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CombinedSheet" sheetId="2" r:id="rId1"/>
-    <sheet name="DADOS" sheetId="3" state="hidden" r:id="rId2"/>
+    <sheet name="Planilha1" sheetId="4" r:id="rId2"/>
+    <sheet name="DADOS" sheetId="3" state="hidden" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">CombinedSheet!$A$1:$Q$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">DADOS!$A$1:$F$352</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">DADOS!$A$1:$F$352</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
   <extLst>
@@ -30,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="29">
   <si>
     <t>UO_COD</t>
   </si>
@@ -238,7 +239,7 @@
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -261,6 +262,12 @@
       <patternFill patternType="solid">
         <fgColor theme="0"/>
         <bgColor theme="0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor rgb="FF000000"/>
       </patternFill>
     </fill>
   </fills>
@@ -388,7 +395,7 @@
     <xf numFmtId="43" fontId="6" fillId="0" borderId="1" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="1" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -437,6 +444,15 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="43" fontId="10" fillId="0" borderId="3" xfId="26" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="11" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -788,74 +804,90 @@
     </row>
     <row r="2" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3">
-        <v>1231</v>
+        <v>1081</v>
       </c>
       <c r="B2" s="3">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C2" s="3">
         <v>0</v>
       </c>
       <c r="D2" s="3">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="E2" s="3">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="F2" s="15">
-        <v>4419</v>
-      </c>
-      <c r="G2" s="15" t="s">
-        <v>28</v>
-      </c>
-      <c r="H2" s="15"/>
-      <c r="I2" s="16"/>
-      <c r="J2" s="17">
-        <v>18380103.300000001</v>
-      </c>
+        <v>7803</v>
+      </c>
+      <c r="G2" s="15"/>
+      <c r="H2" s="15">
+        <v>9116</v>
+      </c>
+      <c r="I2" s="16">
+        <v>7000000</v>
+      </c>
+      <c r="J2" s="17"/>
       <c r="K2" s="2"/>
       <c r="L2" s="2"/>
     </row>
     <row r="3" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="11">
-        <v>1231</v>
+        <v>1081</v>
       </c>
       <c r="B3" s="11">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C3" s="11">
         <v>0</v>
       </c>
       <c r="D3" s="11">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="E3" s="11">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="F3" s="12">
-        <v>4420</v>
-      </c>
-      <c r="G3" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="H3" s="12"/>
-      <c r="I3" s="13"/>
-      <c r="J3" s="14">
-        <v>888800.80999999994</v>
-      </c>
+        <v>7803</v>
+      </c>
+      <c r="G3" s="12"/>
+      <c r="H3" s="12">
+        <v>9103</v>
+      </c>
+      <c r="I3" s="13">
+        <v>10000000</v>
+      </c>
+      <c r="J3" s="14"/>
       <c r="K3" s="2"/>
       <c r="L3" s="2"/>
     </row>
     <row r="4" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="3"/>
-      <c r="B4" s="3"/>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
-      <c r="E4" s="3"/>
-      <c r="F4" s="2"/>
+      <c r="A4" s="3">
+        <v>1081</v>
+      </c>
+      <c r="B4" s="3">
+        <v>3</v>
+      </c>
+      <c r="C4" s="3">
+        <v>0</v>
+      </c>
+      <c r="D4" s="3">
+        <v>10</v>
+      </c>
+      <c r="E4" s="3">
+        <v>9</v>
+      </c>
+      <c r="F4" s="2">
+        <v>7803</v>
+      </c>
       <c r="G4" s="2"/>
-      <c r="H4" s="2"/>
-      <c r="I4" s="7"/>
+      <c r="H4" s="2">
+        <v>1310</v>
+      </c>
+      <c r="I4" s="7">
+        <v>3000000</v>
+      </c>
       <c r="J4" s="4"/>
       <c r="K4" s="2"/>
       <c r="L4" s="2"/>
@@ -866,15 +898,31 @@
       <c r="Q4" s="8"/>
     </row>
     <row r="5" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="3"/>
-      <c r="B5" s="3"/>
-      <c r="C5" s="3"/>
-      <c r="D5" s="3"/>
-      <c r="E5" s="3"/>
-      <c r="F5" s="2"/>
+      <c r="A5" s="3">
+        <v>1081</v>
+      </c>
+      <c r="B5" s="3">
+        <v>1</v>
+      </c>
+      <c r="C5" s="3">
+        <v>0</v>
+      </c>
+      <c r="D5" s="3">
+        <v>10</v>
+      </c>
+      <c r="E5" s="3">
+        <v>9</v>
+      </c>
+      <c r="F5" s="2">
+        <v>7803</v>
+      </c>
       <c r="G5" s="2"/>
-      <c r="H5" s="2"/>
-      <c r="I5" s="7"/>
+      <c r="H5" s="2">
+        <v>9103</v>
+      </c>
+      <c r="I5" s="7">
+        <v>10000000</v>
+      </c>
       <c r="J5" s="4"/>
       <c r="K5" s="2"/>
       <c r="L5" s="2"/>
@@ -8232,6 +8280,43 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{905606C8-2DA6-4405-B9A4-3DDB09CD6E91}">
+  <dimension ref="A1:I1"/>
+  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:9" ht="15" x14ac:dyDescent="0.25">
+      <c r="A1" s="18">
+        <v>1261</v>
+      </c>
+      <c r="B1" s="18">
+        <v>3</v>
+      </c>
+      <c r="C1" s="18">
+        <v>0</v>
+      </c>
+      <c r="D1" s="18">
+        <v>10</v>
+      </c>
+      <c r="E1" s="18">
+        <v>1</v>
+      </c>
+      <c r="F1" s="19">
+        <v>2122</v>
+      </c>
+      <c r="G1" s="19" t="s">
+        <v>28</v>
+      </c>
+      <c r="H1" s="19"/>
+      <c r="I1" s="20">
+        <v>3571806.82</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:F353"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
@@ -10398,6 +10483,17 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="b91e7f20-fe0a-487d-91a9-605ac1c64acf" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="6f4338ef-addb-4c87-aefe-1895241b335f">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100B08D58FADB61F04EBBB4F355C06EFBED" ma:contentTypeVersion="19" ma:contentTypeDescription="Crie um novo documento." ma:contentTypeScope="" ma:versionID="b1e0f6055e0e9a4b9e75d6c71ee7de91">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="6f4338ef-addb-4c87-aefe-1895241b335f" xmlns:ns3="b91e7f20-fe0a-487d-91a9-605ac1c64acf" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="b43930f3490e4d4da1ab3f8da7df6f51" ns2:_="" ns3:_="">
     <xsd:import namespace="6f4338ef-addb-4c87-aefe-1895241b335f"/>
@@ -10658,7 +10754,7 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
@@ -10667,18 +10763,18 @@
 </FormTemplates>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="b91e7f20-fe0a-487d-91a9-605ac1c64acf" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="6f4338ef-addb-4c87-aefe-1895241b335f">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{78AD39BD-2F37-414E-8652-4DCF45E4F24B}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="b91e7f20-fe0a-487d-91a9-605ac1c64acf"/>
+    <ds:schemaRef ds:uri="6f4338ef-addb-4c87-aefe-1895241b335f"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9E3F47A8-3F3E-4CD4-856C-EFC2EF6F2BBF}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -10697,21 +10793,10 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A11A0DA3-0444-476A-A216-870D1067E696}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{78AD39BD-2F37-414E-8652-4DCF45E4F24B}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="b91e7f20-fe0a-487d-91a9-605ac1c64acf"/>
-    <ds:schemaRef ds:uri="6f4338ef-addb-4c87-aefe-1895241b335f"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
feat: reescreve consolida.py e ajusta fluxo_aprovar e cota_orcamentaria
consolida.py: logica completa de consolidacao do arquivo de conferencia
com suporte a multiplas execucoes no mesmo dia (campo Execucao), uso de
ONEDRIVE_BASE do .env e movimentacao correta entre pastas
fluxo_aprovar.py: ajuste pontual no fluxo
cota_orcamentaria.py: melhorias no modulo de cota

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/remanejamento.xlsx
+++ b/data/remanejamento.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\guilhermemelof\code\splor-mg\siafi-automacao-cota\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\brunohorosa\code\splor-mg\siafi-automacao-cota\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B4C85F4-DE41-4A33-B9A0-48623C19BC30}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FCC5A4A7-CD64-403F-A0EB-C7F6C0A33E69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CombinedSheet" sheetId="2" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="29">
   <si>
     <t>UO_COD</t>
   </si>
@@ -129,7 +129,7 @@
     <numFmt numFmtId="164" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* \-??_);_(@_)"/>
     <numFmt numFmtId="165" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@"/>
   </numFmts>
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="17" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -219,11 +219,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -239,7 +234,7 @@
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -256,12 +251,6 @@
       <patternFill patternType="solid">
         <fgColor theme="4" tint="0.39997558519241921"/>
         <bgColor rgb="FF953734"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="0"/>
-        <bgColor theme="0"/>
       </patternFill>
     </fill>
     <fill>
@@ -395,7 +384,7 @@
     <xf numFmtId="43" fontId="6" fillId="0" borderId="1" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="1" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -425,16 +414,13 @@
     <xf numFmtId="10" fontId="12" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="1" fontId="14" fillId="4" borderId="4" xfId="34" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="4" xfId="34" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="4" xfId="34" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="15" fillId="0" borderId="5" xfId="34" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="165" fontId="16" fillId="0" borderId="5" xfId="34" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="17" fillId="0" borderId="5" xfId="34" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="33" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -446,7 +432,7 @@
     <xf numFmtId="43" fontId="10" fillId="0" borderId="3" xfId="26" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -804,7 +790,7 @@
     </row>
     <row r="2" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3">
-        <v>1081</v>
+        <v>1261</v>
       </c>
       <c r="B2" s="3">
         <v>3</v>
@@ -816,78 +802,62 @@
         <v>10</v>
       </c>
       <c r="E2" s="3">
-        <v>9</v>
-      </c>
-      <c r="F2" s="15">
-        <v>7803</v>
-      </c>
-      <c r="G2" s="15"/>
-      <c r="H2" s="15">
-        <v>9116</v>
-      </c>
-      <c r="I2" s="16">
-        <v>7000000</v>
-      </c>
-      <c r="J2" s="17"/>
+        <v>1</v>
+      </c>
+      <c r="F2" s="14">
+        <v>4547</v>
+      </c>
+      <c r="G2" s="14" t="s">
+        <v>28</v>
+      </c>
+      <c r="H2" s="14"/>
+      <c r="I2" s="15">
+        <v>1</v>
+      </c>
+      <c r="J2" s="16"/>
       <c r="K2" s="2"/>
       <c r="L2" s="2"/>
     </row>
     <row r="3" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="11">
-        <v>1081</v>
-      </c>
-      <c r="B3" s="11">
+      <c r="A3" s="3">
+        <v>1261</v>
+      </c>
+      <c r="B3" s="3">
         <v>3</v>
       </c>
-      <c r="C3" s="11">
+      <c r="C3" s="3">
         <v>0</v>
       </c>
-      <c r="D3" s="11">
+      <c r="D3" s="3">
         <v>10</v>
       </c>
-      <c r="E3" s="11">
-        <v>9</v>
-      </c>
-      <c r="F3" s="12">
-        <v>7803</v>
-      </c>
-      <c r="G3" s="12"/>
-      <c r="H3" s="12">
-        <v>9103</v>
-      </c>
-      <c r="I3" s="13">
-        <v>10000000</v>
-      </c>
-      <c r="J3" s="14"/>
+      <c r="E3" s="3">
+        <v>1</v>
+      </c>
+      <c r="F3" s="14">
+        <v>4547</v>
+      </c>
+      <c r="G3" s="14" t="s">
+        <v>28</v>
+      </c>
+      <c r="H3" s="11"/>
+      <c r="I3" s="12"/>
+      <c r="J3" s="13">
+        <v>1</v>
+      </c>
       <c r="K3" s="2"/>
       <c r="L3" s="2"/>
     </row>
     <row r="4" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="3">
-        <v>1081</v>
-      </c>
-      <c r="B4" s="3">
-        <v>3</v>
-      </c>
-      <c r="C4" s="3">
-        <v>0</v>
-      </c>
-      <c r="D4" s="3">
-        <v>10</v>
-      </c>
-      <c r="E4" s="3">
-        <v>9</v>
-      </c>
-      <c r="F4" s="2">
-        <v>7803</v>
-      </c>
+      <c r="A4" s="3"/>
+      <c r="B4" s="3"/>
+      <c r="C4" s="3"/>
+      <c r="D4" s="3"/>
+      <c r="E4" s="3"/>
+      <c r="F4" s="2"/>
       <c r="G4" s="2"/>
-      <c r="H4" s="2">
-        <v>1310</v>
-      </c>
-      <c r="I4" s="7">
-        <v>3000000</v>
-      </c>
+      <c r="H4" s="2"/>
+      <c r="I4" s="7"/>
       <c r="J4" s="4"/>
       <c r="K4" s="2"/>
       <c r="L4" s="2"/>
@@ -898,31 +868,15 @@
       <c r="Q4" s="8"/>
     </row>
     <row r="5" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="3">
-        <v>1081</v>
-      </c>
-      <c r="B5" s="3">
-        <v>1</v>
-      </c>
-      <c r="C5" s="3">
-        <v>0</v>
-      </c>
-      <c r="D5" s="3">
-        <v>10</v>
-      </c>
-      <c r="E5" s="3">
-        <v>9</v>
-      </c>
-      <c r="F5" s="2">
-        <v>7803</v>
-      </c>
+      <c r="A5" s="3"/>
+      <c r="B5" s="3"/>
+      <c r="C5" s="3"/>
+      <c r="D5" s="3"/>
+      <c r="E5" s="3"/>
+      <c r="F5" s="2"/>
       <c r="G5" s="2"/>
-      <c r="H5" s="2">
-        <v>9103</v>
-      </c>
-      <c r="I5" s="7">
-        <v>10000000</v>
-      </c>
+      <c r="H5" s="2"/>
+      <c r="I5" s="7"/>
       <c r="J5" s="4"/>
       <c r="K5" s="2"/>
       <c r="L5" s="2"/>
@@ -8241,19 +8195,19 @@
           <x14:formula1>
             <xm:f>DADOS!$A$2:$A$82</xm:f>
           </x14:formula1>
-          <xm:sqref>A3:A61</xm:sqref>
+          <xm:sqref>A4:A61</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0000-000002000000}">
           <x14:formula1>
             <xm:f>DADOS!$B$2:$B$3</xm:f>
           </x14:formula1>
-          <xm:sqref>C3:C61</xm:sqref>
+          <xm:sqref>C4:C61</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0000-000003000000}">
           <x14:formula1>
             <xm:f>DADOS!$E$2:$E$5</xm:f>
           </x14:formula1>
-          <xm:sqref>B3:B61</xm:sqref>
+          <xm:sqref>B4:B61</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0000-000005000000}">
           <x14:formula1>
@@ -8265,13 +8219,13 @@
           <x14:formula1>
             <xm:f>DADOS!$D$2:$D$5</xm:f>
           </x14:formula1>
-          <xm:sqref>E3:E61</xm:sqref>
+          <xm:sqref>E4:E61</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0000-000007000000}">
           <x14:formula1>
             <xm:f>DADOS!$C$2:$C$32</xm:f>
           </x14:formula1>
-          <xm:sqref>D3:D61</xm:sqref>
+          <xm:sqref>D4:D61</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -8285,29 +8239,29 @@
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:9" ht="15" x14ac:dyDescent="0.25">
-      <c r="A1" s="18">
+      <c r="A1" s="17">
         <v>1261</v>
       </c>
-      <c r="B1" s="18">
+      <c r="B1" s="17">
         <v>3</v>
       </c>
-      <c r="C1" s="18">
+      <c r="C1" s="17">
         <v>0</v>
       </c>
-      <c r="D1" s="18">
+      <c r="D1" s="17">
         <v>10</v>
       </c>
-      <c r="E1" s="18">
+      <c r="E1" s="17">
         <v>1</v>
       </c>
-      <c r="F1" s="19">
+      <c r="F1" s="18">
         <v>2122</v>
       </c>
-      <c r="G1" s="19" t="s">
+      <c r="G1" s="18" t="s">
         <v>28</v>
       </c>
-      <c r="H1" s="19"/>
-      <c r="I1" s="20">
+      <c r="H1" s="18"/>
+      <c r="I1" s="19">
         <v>3571806.82</v>
       </c>
     </row>
@@ -10483,17 +10437,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="b91e7f20-fe0a-487d-91a9-605ac1c64acf" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="6f4338ef-addb-4c87-aefe-1895241b335f">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100B08D58FADB61F04EBBB4F355C06EFBED" ma:contentTypeVersion="19" ma:contentTypeDescription="Crie um novo documento." ma:contentTypeScope="" ma:versionID="b1e0f6055e0e9a4b9e75d6c71ee7de91">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="6f4338ef-addb-4c87-aefe-1895241b335f" xmlns:ns3="b91e7f20-fe0a-487d-91a9-605ac1c64acf" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="b43930f3490e4d4da1ab3f8da7df6f51" ns2:_="" ns3:_="">
     <xsd:import namespace="6f4338ef-addb-4c87-aefe-1895241b335f"/>
@@ -10754,6 +10697,17 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="b91e7f20-fe0a-487d-91a9-605ac1c64acf" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="6f4338ef-addb-4c87-aefe-1895241b335f">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -10764,17 +10718,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{78AD39BD-2F37-414E-8652-4DCF45E4F24B}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="b91e7f20-fe0a-487d-91a9-605ac1c64acf"/>
-    <ds:schemaRef ds:uri="6f4338ef-addb-4c87-aefe-1895241b335f"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9E3F47A8-3F3E-4CD4-856C-EFC2EF6F2BBF}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -10793,6 +10736,17 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{78AD39BD-2F37-414E-8652-4DCF45E4F24B}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="b91e7f20-fe0a-487d-91a9-605ac1c64acf"/>
+    <ds:schemaRef ds:uri="6f4338ef-addb-4c87-aefe-1895241b335f"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A11A0DA3-0444-476A-A216-870D1067E696}">
   <ds:schemaRefs>

</xml_diff>